<commit_message>
Day 15 with updates
</commit_message>
<xml_diff>
--- a/Day-10/rejected_students.xlsx
+++ b/Day-10/rejected_students.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,6 +458,19 @@
         <v>78</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rohit</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C3" t="n">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>